<commit_message>
I will check the current status of the repository and the recent commit history to ensure the message is consistent with the project's style. I will use the generalist agent to check the current repository status and commit history. I will generate a git commit message based on the provided diff, noting the update to the network test tracing documentation and the removal of the temporary lock file.
```text
docs: update Connectivity Room Network Test Tracing System document

- Update docs/Connectivity Room Network Test Tracing System.xlsx
- Remove temporary Excel lock file
```
</commit_message>
<xml_diff>
--- a/docs/Connectivity Room Network Test Tracing System.xlsx
+++ b/docs/Connectivity Room Network Test Tracing System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\product_test_tracing_system\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D661DD4-AC08-4268-8799-3C63FE969061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E6F426-8BF0-49C8-911E-9D4CC5096FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="745" firstSheet="5" activeTab="5" xr2:uid="{421B0B10-1399-475F-B14E-2C2D39CF6739}"/>
   </bookViews>
@@ -35,6 +35,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Connectivity Room Routers'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Connectivity Room Routers (2)'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Cases (2)'!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3687" uniqueCount="587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3708" uniqueCount="665">
   <si>
     <t>HRK-9000A</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2698,6 +2699,9 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>Test Config ID</t>
+  </si>
+  <si>
     <t>Test Case ID(PK)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -2716,11 +2720,559 @@
   </si>
   <si>
     <t>CONFIG_ID</t>
+  </si>
+  <si>
+    <t>CONFIG_ID</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>설정명</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>시험환경별칭</t>
+  </si>
+  <si>
+    <t>시험대상</t>
+  </si>
+  <si>
+    <t>시험환경</t>
+  </si>
+  <si>
+    <t>시험조건</t>
+  </si>
+  <si>
+    <t>CFG-HRK-WIFI-AP_2_4G-001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TBD(To Be Determind, 협의사항)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>결정사항</t>
+  </si>
+  <si>
+    <t>테스트대상 구성 (장비 대수, S/W Version): 
+- HRK-9000A (1대, 1.01.01A)
+테스트환경 구성 : 
+- AP(2.4GHz Band) 1대
+- HDR-9000 1대</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1.01.01A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TEST_RELEASE_ID-HRK-9000A_1.01.01A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TBD(To Be Determined, 협의사항)</t>
+  </si>
+  <si>
+    <t>시험환경구성절차_재현판단기준</t>
+  </si>
+  <si>
+    <t>1. TBD(Wireless / Channel)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. TBD(Channel Width / Bandwidth)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. TBD(Wireless Mode)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. TBD(WPA2-보안)
+2. Personal
+3. AES</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>시험환경구성절차</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SQA HRK Wi-Fi 2.4GHz Router 단독 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HRK Wi-Fi 2.4GHz Router + HDR 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HLM Wi-Fi 2.4GHz Router 단독 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HLM Wi-Fi 2.4GHz Router + HDR 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HTR Wi-Fi 2.4GHz Router 단독 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HTR Wi-Fi 2.4GHz Router + HDR 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDR Wi-Fi 2.4GHz Router 단독 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDR Wi-Fi 2.4GHz Router + HRK 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDR Wi-Fi 2.4GHz Router + HLM 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDR Wi-Fi 2.4GHz Router + HTR 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDR Wi-Fi 2.4GHz Router + HRK/HLM/HTR 복합 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDR Wi-Fi 2.4GHz Router + HIIS-1 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDR Wi-Fi 2.4GHz Router + HDC 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDC Wi-Fi 2.4GHz Router 단독 환경 구성 01</t>
+  </si>
+  <si>
+    <t>SQA HDC Wi-Fi 2.4GHz Router + HDR 연동 환경 구성 01</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: 없음_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HRK 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: 없음_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HLM 전원 공급용 케이블: AC 전원 공급용 케이블(L-형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: 없음_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HTR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: 없음_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HRK-9000A 1대_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - HRK 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HLM-9000 1대_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - HLM 전원 공급용 케이블: AC 전원 공급용 케이블(L-형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HTR-TODO 1대_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - HTR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HRK-9000A 1대, HLM-9000 1대, HTR-TODO 1대_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - HRK 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HLM 전원 공급용 케이블: AC 전원 공급용 케이블(L-형)_x000D_
+  - HTR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HIIS-1 1대_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HDC-9100 1대_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - HDC 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: 없음_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDC 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>Router Test Case Procedure</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AP 설정 및 구성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HRK-9000A-WIFI-ROUTER_2_4G-001</t>
+  </si>
+  <si>
+    <t>[시험대상]_x000D_
+- 시험대상_제조사: Huvitz_x000D_
+- 시험대상_제품명: HRK-9000A_x000D_
+- 수량: 1대</t>
+  </si>
+  <si>
+    <t>[시험조건]_x000D_
+- Router Wi-Fi Band: 2.4GHz_x000D_
+- Router Wi-Fi SSID: xxxxxx_2_4G_x000D_
+- Router Wi-Fi Channel: TBD_x000D_
+- Router Channel Bandwidth: TBD_x000D_
+- Router Wireless Mode: TBD_x000D_
+- Router Security Mode: TBD_x000D_
+- Router Encryption: TBD_x000D_
+- Router 와 시험대상 간 거리: TBD</t>
+  </si>
+  <si>
+    <t>TBD : 렌즈 측정 모의용 장치 사양 지정 필요_x000D_
+TBD : 눈 검사 모의용 장치 모델명 지정 필요_x000D_
+TBD : Router Wi-Fi SSID 설정완료확인방법 지정 필요_x000D_
+- Smart Connect 옵션: (Off)_x000D_
+- Band Steering 옵션: (Off)_x000D_
+TBD : Router Wi-Fi Channel 및 설정완료확인방법 지정 필요_x000D_
+- 2.4GHz Channel 옵션: (1|6|11)_x000D_
+- 5GHz Channel 옵션: (36|40|44|48)_x000D_
+TBD : Router Channel Bandwidth 및 설정완료확인방법 지정 필요_x000D_
+- Channel Bandwidth 옵션: (20MHz)_x000D_
+TBD : Router Wi-Fi Wireless Mode 및 설정완료확인방법 지정 필요_x000D_
+- Wireless Mode 옵션: (802.11 b/g/n mixed|802.11 a/b/g/n mixed)_x000D_
+TBD : Router Wi-Fi Security 및 설정완료확인방법 지정 필요_x000D_
+- Security 옵션: (WPA2|WPA2-Personal)_x000D_
+- Encryption 옵션: (AES)_x000D_
+TBD : Router 와 시험대상 간 거리 지정 필요_x000D_
+- 거리 옵션: (1m|3m|5m|TBD)</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HRK-9000A-WIFI-ROUTER_2_4G-HDR-9000-001</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HDR-9000 1대_x000D_
+- 연동장비_구성요소: HDR-9000_OP, HDR-9000_JUNCTION_BOX, HDR-9000_TODO_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HRK 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>TBD : 연동장비_구성요소 HDR-9000_TODO 확정 필요_x000D_
+TBD : 렌즈 측정 모의용 장치 사양 지정 필요_x000D_
+TBD : 눈 검사 모의용 장치 모델명 지정 필요_x000D_
+TBD : Router Wi-Fi SSID 설정완료확인방법 지정 필요_x000D_
+- Smart Connect 옵션: (Off)_x000D_
+- Band Steering 옵션: (Off)_x000D_
+TBD : Router Wi-Fi Channel 및 설정완료확인방법 지정 필요_x000D_
+- 2.4GHz Channel 옵션: (1|6|11)_x000D_
+- 5GHz Channel 옵션: (36|40|44|48)_x000D_
+TBD : Router Channel Bandwidth 및 설정완료확인방법 지정 필요_x000D_
+- Channel Bandwidth 옵션: (20MHz)_x000D_
+TBD : Router Wi-Fi Wireless Mode 및 설정완료확인방법 지정 필요_x000D_
+- Wireless Mode 옵션: (802.11 b/g/n mixed|802.11 a/b/g/n mixed)_x000D_
+TBD : Router Wi-Fi Security 및 설정완료확인방법 지정 필요_x000D_
+- Security 옵션: (WPA2|WPA2-Personal)_x000D_
+- Encryption 옵션: (AES)_x000D_
+TBD : Router 와 시험대상 간 거리 지정 필요_x000D_
+- 거리 옵션: (1m|3m|5m|TBD)</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HLM-9000-WIFI-ROUTER_2_4G-001</t>
+  </si>
+  <si>
+    <t>[시험대상]_x000D_
+- 시험대상_제조사: Huvitz_x000D_
+- 시험대상_제품명: HLM-9000_x000D_
+- 수량: 1대</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HLM-9000-WIFI-ROUTER_2_4G-HDR-9000-001</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HDR-9000 1대_x000D_
+- 연동장비_구성요소: HDR-9000_OP, HDR-9000_JUNCTION_BOX, HDR-9000_TODO_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HLM 전원 공급용 케이블: AC 전원 공급용 케이블(L-형)_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HTR-TODO-WIFI-ROUTER_2_4G-001</t>
+  </si>
+  <si>
+    <t>[시험대상]_x000D_
+- 시험대상_제조사: Huvitz_x000D_
+- 시험대상_제품명: HTR-TODO_x000D_
+- 수량: 1대</t>
+  </si>
+  <si>
+    <t>TBD : 시험대상_제품명 HTR-TODO 확정 필요_x000D_
+TBD : 렌즈 측정 모의용 장치 사양 지정 필요_x000D_
+TBD : 눈 검사 모의용 장치 모델명 지정 필요_x000D_
+TBD : Router Wi-Fi SSID 설정완료확인방법 지정 필요_x000D_
+- Smart Connect 옵션: (Off)_x000D_
+- Band Steering 옵션: (Off)_x000D_
+TBD : Router Wi-Fi Channel 및 설정완료확인방법 지정 필요_x000D_
+- 2.4GHz Channel 옵션: (1|6|11)_x000D_
+- 5GHz Channel 옵션: (36|40|44|48)_x000D_
+TBD : Router Channel Bandwidth 및 설정완료확인방법 지정 필요_x000D_
+- Channel Bandwidth 옵션: (20MHz)_x000D_
+TBD : Router Wi-Fi Wireless Mode 및 설정완료확인방법 지정 필요_x000D_
+- Wireless Mode 옵션: (802.11 b/g/n mixed|802.11 a/b/g/n mixed)_x000D_
+TBD : Router Wi-Fi Security 및 설정완료확인방법 지정 필요_x000D_
+- Security 옵션: (WPA2|WPA2-Personal)_x000D_
+- Encryption 옵션: (AES)_x000D_
+TBD : Router 와 시험대상 간 거리 지정 필요_x000D_
+- 거리 옵션: (1m|3m|5m|TBD)</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HTR-TODO-WIFI-ROUTER_2_4G-HDR-9000-001</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HDR-9000 1대_x000D_
+- 연동장비_구성요소: HDR-9000_OP, HDR-9000_JUNCTION_BOX, HDR-9000_TODO_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HTR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
+  </si>
+  <si>
+    <t>TBD : 시험대상_제품명 HTR-TODO 확정 필요_x000D_
+TBD : 연동장비_구성요소 HDR-9000_TODO 확정 필요_x000D_
+TBD : 렌즈 측정 모의용 장치 사양 지정 필요_x000D_
+TBD : 눈 검사 모의용 장치 모델명 지정 필요_x000D_
+TBD : Router Wi-Fi SSID 설정완료확인방법 지정 필요_x000D_
+- Smart Connect 옵션: (Off)_x000D_
+- Band Steering 옵션: (Off)_x000D_
+TBD : Router Wi-Fi Channel 및 설정완료확인방법 지정 필요_x000D_
+- 2.4GHz Channel 옵션: (1|6|11)_x000D_
+- 5GHz Channel 옵션: (36|40|44|48)_x000D_
+TBD : Router Channel Bandwidth 및 설정완료확인방법 지정 필요_x000D_
+- Channel Bandwidth 옵션: (20MHz)_x000D_
+TBD : Router Wi-Fi Wireless Mode 및 설정완료확인방법 지정 필요_x000D_
+- Wireless Mode 옵션: (802.11 b/g/n mixed|802.11 a/b/g/n mixed)_x000D_
+TBD : Router Wi-Fi Security 및 설정완료확인방법 지정 필요_x000D_
+- Security 옵션: (WPA2|WPA2-Personal)_x000D_
+- Encryption 옵션: (AES)_x000D_
+TBD : Router 와 시험대상 간 거리 지정 필요_x000D_
+- 거리 옵션: (1m|3m|5m|TBD)</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDR-9000-WIFI-ROUTER_2_4G-001</t>
+  </si>
+  <si>
+    <t>[시험대상]_x000D_
+- 시험대상_제조사: Huvitz_x000D_
+- 시험대상_제품명: HDR-9000_x000D_
+- 시험대상_구성요소: HDR-9000_OP, HDR-9000_JUNCTION_BOX, HDR-9000_TODO_x000D_
+- 수량: 1대</t>
+  </si>
+  <si>
+    <t>TBD : 시험대상_구성요소 HDR-9000_TODO 확정 필요_x000D_
+TBD : 렌즈 측정 모의용 장치 사양 지정 필요_x000D_
+TBD : 눈 검사 모의용 장치 모델명 지정 필요_x000D_
+TBD : Router Wi-Fi SSID 설정완료확인방법 지정 필요_x000D_
+- Smart Connect 옵션: (Off)_x000D_
+- Band Steering 옵션: (Off)_x000D_
+TBD : Router Wi-Fi Channel 및 설정완료확인방법 지정 필요_x000D_
+- 2.4GHz Channel 옵션: (1|6|11)_x000D_
+- 5GHz Channel 옵션: (36|40|44|48)_x000D_
+TBD : Router Channel Bandwidth 및 설정완료확인방법 지정 필요_x000D_
+- Channel Bandwidth 옵션: (20MHz)_x000D_
+TBD : Router Wi-Fi Wireless Mode 및 설정완료확인방법 지정 필요_x000D_
+- Wireless Mode 옵션: (802.11 b/g/n mixed|802.11 a/b/g/n mixed)_x000D_
+TBD : Router Wi-Fi Security 및 설정완료확인방법 지정 필요_x000D_
+- Security 옵션: (WPA2|WPA2-Personal)_x000D_
+- Encryption 옵션: (AES)_x000D_
+TBD : Router 와 시험대상 간 거리 지정 필요_x000D_
+- 거리 옵션: (1m|3m|5m|TBD)</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDR-9000-WIFI-ROUTER_2_4G-HRK-9000A-001</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDR-9000-WIFI-ROUTER_2_4G-HLM-9000-001</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDR-9000-WIFI-ROUTER_2_4G-HTR-TODO-001</t>
+  </si>
+  <si>
+    <t>TBD : 시험대상_구성요소 HDR-9000_TODO 확정 필요_x000D_
+TBD : 연동장비 HTR-TODO 정식 제품명 확정 필요_x000D_
+TBD : 렌즈 측정 모의용 장치 사양 지정 필요_x000D_
+TBD : 눈 검사 모의용 장치 모델명 지정 필요_x000D_
+TBD : Router Wi-Fi SSID 설정완료확인방법 지정 필요_x000D_
+- Smart Connect 옵션: (Off)_x000D_
+- Band Steering 옵션: (Off)_x000D_
+TBD : Router Wi-Fi Channel 및 설정완료확인방법 지정 필요_x000D_
+- 2.4GHz Channel 옵션: (1|6|11)_x000D_
+- 5GHz Channel 옵션: (36|40|44|48)_x000D_
+TBD : Router Channel Bandwidth 및 설정완료확인방법 지정 필요_x000D_
+- Channel Bandwidth 옵션: (20MHz)_x000D_
+TBD : Router Wi-Fi Wireless Mode 및 설정완료확인방법 지정 필요_x000D_
+- Wireless Mode 옵션: (802.11 b/g/n mixed|802.11 a/b/g/n mixed)_x000D_
+TBD : Router Wi-Fi Security 및 설정완료확인방법 지정 필요_x000D_
+- Security 옵션: (WPA2|WPA2-Personal)_x000D_
+- Encryption 옵션: (AES)_x000D_
+TBD : Router 와 시험대상 간 거리 지정 필요_x000D_
+- 거리 옵션: (1m|3m|5m|TBD)</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDR-9000-WIFI-ROUTER_2_4G-HRK-9000A-HLM-9000-HTR-TODO-001</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDR-9000-WIFI-ROUTER_2_4G-HIIS-1-001</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDR-9000-WIFI-ROUTER_2_4G-HDC-9100-001</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDC-9100-WIFI-ROUTER_2_4G-001</t>
+  </si>
+  <si>
+    <t>[시험대상]_x000D_
+- 시험대상_제조사: Huvitz_x000D_
+- 시험대상_제품명: HDC-9100_x000D_
+- 수량: 1대</t>
+  </si>
+  <si>
+    <t>SQA_TEST_CONFIG-HDC-9100-WIFI-ROUTER_2_4G-HDR-9000-001</t>
+  </si>
+  <si>
+    <t>[시험환경]_x000D_
+- 시험장소: Huvitz Connectivity Room_x000D_
+- 네트워크유형: Wi-Fi_x000D_
+- Router 구성: MR30G 1대_x000D_
+- Router 제조사: MERCUSYS_x000D_
+- 연동장비: HDR-9000 1대_x000D_
+- 연동장비_구성요소: HDR-9000_OP, HDR-9000_JUNCTION_BOX, HDR-9000_TODO_x000D_
+- 연동보조장비/케이블:_x000D_
+  - HDC 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 공급용 케이블: AC 전원 공급용 케이블(직선형)_x000D_
+  - HDR 전원 및 신호 공급용 케이블: OP Signal and Power Cable_x000D_
+  - HDR 전원 및 신호 공급용 케이블: HDR Signal and Power Cable_x000D_
+  - 렌즈 측정 모의용 장치: Lens TBD(x mm)_x000D_
+  - 눈 검사 모의용 장치: 모델아이 TBD</t>
   </si>
 </sst>
 </file>
@@ -2730,7 +3282,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2825,8 +3377,15 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2854,6 +3413,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
       </patternFill>
     </fill>
   </fills>
@@ -2998,18 +3562,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3184,19 +3751,43 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="2" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="강조색1" xfId="1" builtinId="29"/>
+    <cellStyle name="강조색6" xfId="2" builtinId="49"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="하이퍼링크" xfId="2" builtinId="8"/>
+    <cellStyle name="하이퍼링크" xfId="3" builtinId="8"/>
   </cellStyles>
-  <dxfs count="89">
+  <dxfs count="91">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -4153,7 +4744,7 @@
         <v>574</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -4550,47 +5141,47 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="B1:B21">
-    <cfRule type="containsText" dxfId="88" priority="16" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="90" priority="16" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",B1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A21">
-    <cfRule type="containsText" dxfId="87" priority="15" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="89" priority="15" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="containsText" dxfId="86" priority="7" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="88" priority="7" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A25:C45">
-    <cfRule type="containsText" dxfId="85" priority="11" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="87" priority="11" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A25)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="containsText" dxfId="84" priority="5" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="86" priority="5" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",B49)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C49">
-    <cfRule type="containsText" dxfId="83" priority="4" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="85" priority="4" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",C49)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D49">
-    <cfRule type="containsText" dxfId="82" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="84" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D49)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A49">
-    <cfRule type="containsText" dxfId="81" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="83" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A49)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="containsText" dxfId="80" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="82" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4936,7 +5527,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A8:D8">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="36" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A8)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8452,27 +9043,27 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:E26 A43:E50 E35:E42 G35:K50 G1:K26">
-    <cfRule type="containsText" dxfId="61" priority="5" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="35" priority="5" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:E27 B28:E34 G27:K34">
-    <cfRule type="containsText" dxfId="60" priority="4" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="34" priority="4" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F26 F43:F50">
-    <cfRule type="containsText" dxfId="59" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="33" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F27">
-    <cfRule type="containsText" dxfId="58" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="32" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="containsText" dxfId="57" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="31" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11402,17 +11993,17 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:E19 G1:K19">
-    <cfRule type="containsText" dxfId="56" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F19">
-    <cfRule type="containsText" dxfId="55" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="containsText" dxfId="54" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14458,17 +15049,17 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:E23 G1:K23">
-    <cfRule type="containsText" dxfId="53" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="27" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F23">
-    <cfRule type="containsText" dxfId="52" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="26" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="containsText" dxfId="51" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="25" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17520,17 +18111,17 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:E26 G1:K26">
-    <cfRule type="containsText" dxfId="50" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="24" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F26">
-    <cfRule type="containsText" dxfId="49" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="23" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="containsText" dxfId="48" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="22" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20558,22 +21149,22 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:E27 G1:K27">
-    <cfRule type="containsText" dxfId="47" priority="5" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="21" priority="5" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2 F8:F27">
-    <cfRule type="containsText" dxfId="46" priority="4" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="20" priority="4" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="containsText" dxfId="45" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="19" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5">
-    <cfRule type="containsText" dxfId="44" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25155,92 +25746,92 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:E26 A43:E50 E35:E42 G35:K50 G1:K26">
-    <cfRule type="containsText" dxfId="43" priority="18" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="17" priority="18" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:E27 B28:E34 G27:K34">
-    <cfRule type="containsText" dxfId="42" priority="17" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="16" priority="17" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F26 F43:F50">
-    <cfRule type="containsText" dxfId="41" priority="16" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="15" priority="16" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F27">
-    <cfRule type="containsText" dxfId="40" priority="15" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="14" priority="15" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="containsText" dxfId="39" priority="14" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="13" priority="14" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A51:E69 G51:K69">
-    <cfRule type="containsText" dxfId="38" priority="13" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="12" priority="13" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A51)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F52:F69">
-    <cfRule type="containsText" dxfId="37" priority="12" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="11" priority="12" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F52)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F51">
-    <cfRule type="containsText" dxfId="36" priority="11" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F51)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A70:E92 G70:K92">
-    <cfRule type="containsText" dxfId="35" priority="10" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="9" priority="10" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A70)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F71:F92">
-    <cfRule type="containsText" dxfId="34" priority="9" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F71)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F70">
-    <cfRule type="containsText" dxfId="33" priority="8" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F70)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A93:E118 G93:K118">
-    <cfRule type="containsText" dxfId="32" priority="7" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A93)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F94:F118">
-    <cfRule type="containsText" dxfId="31" priority="6" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F94)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F93">
-    <cfRule type="containsText" dxfId="30" priority="5" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F93)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A119:E145 G119:K145">
-    <cfRule type="containsText" dxfId="29" priority="4" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A119)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F120 F126:F145">
-    <cfRule type="containsText" dxfId="28" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F120)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F119">
-    <cfRule type="containsText" dxfId="27" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F119)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F123">
-    <cfRule type="containsText" dxfId="26" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F123)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25559,17 +26150,17 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="D5:D7">
-    <cfRule type="containsText" dxfId="79" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="81" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D3">
-    <cfRule type="containsText" dxfId="78" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="80" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D4">
-    <cfRule type="containsText" dxfId="77" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="79" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D4)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25609,7 +26200,7 @@
         <v>13</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="F1" s="22" t="s">
         <v>408</v>
@@ -30011,62 +30602,62 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:D26 G1:K26 A43:D141 G35:K141">
-    <cfRule type="containsText" dxfId="76" priority="20" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="78" priority="20" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:D27 B28:D34 G27:K34">
-    <cfRule type="containsText" dxfId="75" priority="19" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="77" priority="19" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E26 E43:E50">
-    <cfRule type="containsText" dxfId="74" priority="18" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="76" priority="18" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27">
-    <cfRule type="containsText" dxfId="73" priority="17" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="75" priority="17" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="containsText" dxfId="72" priority="16" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="74" priority="16" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E51:E68">
-    <cfRule type="containsText" dxfId="71" priority="14" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="73" priority="14" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E51)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E69:E90">
-    <cfRule type="containsText" dxfId="70" priority="11" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="72" priority="11" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E69)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E91:E115">
-    <cfRule type="containsText" dxfId="69" priority="8" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="71" priority="8" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E91)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E116 E122:E141">
-    <cfRule type="containsText" dxfId="68" priority="5" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="70" priority="5" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E116)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E119">
-    <cfRule type="containsText" dxfId="67" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="69" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E119)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F26 F35:F141">
-    <cfRule type="containsText" dxfId="66" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="68" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F27:F34">
-    <cfRule type="containsText" dxfId="65" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="67" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F27)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -30096,10 +30687,10 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="20" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="C1" s="20" t="s">
         <v>402</v>
@@ -30325,7 +30916,7 @@
       <c r="F10" s="12"/>
       <c r="G10" s="26"/>
       <c r="H10" s="13" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I10" s="13" t="s">
         <v>557</v>
@@ -30643,7 +31234,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:B2 C1:L21">
-    <cfRule type="containsText" dxfId="64" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="66" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -30990,7 +31581,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A8:D8">
-    <cfRule type="containsText" dxfId="62" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="64" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A8)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -31004,574 +31595,722 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D987AB8-9EE7-4A35-B08E-6B0C9A89D789}">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultColWidth="17.5" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="38" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.08203125" customWidth="1"/>
-    <col min="4" max="4" width="31.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.75" customWidth="1"/>
-    <col min="7" max="7" width="28" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.83203125" customWidth="1"/>
+    <col min="1" max="1" width="60.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="68" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.58203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.4140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="41.5" customWidth="1"/>
+    <col min="10" max="10" width="58.4140625" customWidth="1"/>
     <col min="11" max="11" width="60.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="49.33203125" customWidth="1"/>
+    <col min="14" max="14" width="26.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" s="60" t="s">
+        <v>582</v>
+      </c>
+      <c r="B1" s="60" t="s">
+        <v>589</v>
+      </c>
+      <c r="C1" s="60" t="s">
+        <v>590</v>
+      </c>
+      <c r="D1" s="60" t="s">
+        <v>591</v>
+      </c>
+      <c r="E1" s="60" t="s">
+        <v>592</v>
+      </c>
+      <c r="F1" s="60" t="s">
+        <v>599</v>
+      </c>
+      <c r="G1" s="60" t="s">
+        <v>595</v>
+      </c>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+    </row>
+    <row r="2" spans="1:11" ht="164" customHeight="1">
+      <c r="A2" s="62" t="s">
+        <v>634</v>
+      </c>
+      <c r="B2" s="62" t="s">
+        <v>606</v>
+      </c>
+      <c r="C2" s="36" t="s">
+        <v>635</v>
+      </c>
+      <c r="D2" s="36" t="s">
+        <v>621</v>
+      </c>
+      <c r="E2" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F2" s="36" t="s">
+        <v>637</v>
+      </c>
+      <c r="G2" s="36"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+    </row>
+    <row r="3" spans="1:11" ht="247" customHeight="1">
+      <c r="A3" s="62" t="s">
+        <v>638</v>
+      </c>
+      <c r="B3" s="62" t="s">
+        <v>607</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>635</v>
+      </c>
+      <c r="D3" s="36" t="s">
+        <v>639</v>
+      </c>
+      <c r="E3" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F3" s="36" t="s">
+        <v>640</v>
+      </c>
+      <c r="G3" s="36"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+    </row>
+    <row r="4" spans="1:11" ht="79" customHeight="1">
+      <c r="A4" s="62" t="s">
+        <v>641</v>
+      </c>
+      <c r="B4" s="62" t="s">
+        <v>608</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>642</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>622</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F4" s="36" t="s">
+        <v>637</v>
+      </c>
+      <c r="G4" s="36"/>
+      <c r="H4" s="37"/>
+      <c r="I4" s="37"/>
+      <c r="J4" s="37"/>
+      <c r="K4" s="37"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="62" t="s">
+        <v>643</v>
+      </c>
+      <c r="B5" s="62" t="s">
+        <v>609</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>642</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>644</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F5" s="36" t="s">
+        <v>640</v>
+      </c>
+      <c r="G5" s="36"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="62" t="s">
+        <v>645</v>
+      </c>
+      <c r="B6" s="62" t="s">
+        <v>610</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>646</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>623</v>
+      </c>
+      <c r="E6" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F6" s="36" t="s">
+        <v>647</v>
+      </c>
+      <c r="G6" s="36"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="62" t="s">
+        <v>648</v>
+      </c>
+      <c r="B7" s="62" t="s">
+        <v>611</v>
+      </c>
+      <c r="C7" s="36" t="s">
+        <v>646</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>649</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F7" s="36" t="s">
+        <v>650</v>
+      </c>
+      <c r="G7" s="36"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="37"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="62" t="s">
+        <v>651</v>
+      </c>
+      <c r="B8" s="62" t="s">
+        <v>612</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>652</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>624</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F8" s="36" t="s">
+        <v>653</v>
+      </c>
+      <c r="G8" s="36"/>
+      <c r="H8" s="37"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="37"/>
+      <c r="K8" s="37"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="62" t="s">
+        <v>654</v>
+      </c>
+      <c r="B9" s="62" t="s">
+        <v>613</v>
+      </c>
+      <c r="C9" s="36" t="s">
+        <v>652</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>625</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F9" s="36" t="s">
+        <v>653</v>
+      </c>
+      <c r="G9" s="36"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="62" t="s">
+        <v>655</v>
+      </c>
+      <c r="B10" s="62" t="s">
+        <v>614</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>652</v>
+      </c>
+      <c r="D10" s="36" t="s">
+        <v>626</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F10" s="36" t="s">
+        <v>653</v>
+      </c>
+      <c r="G10" s="36"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="37"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="62" t="s">
+        <v>656</v>
+      </c>
+      <c r="B11" s="62" t="s">
+        <v>615</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>652</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>627</v>
+      </c>
+      <c r="E11" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F11" s="36" t="s">
+        <v>657</v>
+      </c>
+      <c r="G11" s="36"/>
+      <c r="H11" s="37"/>
+      <c r="I11" s="37"/>
+      <c r="J11" s="37"/>
+      <c r="K11" s="37"/>
+    </row>
+    <row r="12" spans="1:11" ht="323.5" customHeight="1">
+      <c r="A12" s="62" t="s">
+        <v>658</v>
+      </c>
+      <c r="B12" s="62" t="s">
+        <v>616</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>652</v>
+      </c>
+      <c r="D12" s="36" t="s">
+        <v>628</v>
+      </c>
+      <c r="E12" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F12" s="36" t="s">
+        <v>657</v>
+      </c>
+      <c r="G12" s="36"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="62" t="s">
+        <v>659</v>
+      </c>
+      <c r="B13" s="62" t="s">
+        <v>617</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>652</v>
+      </c>
+      <c r="D13" s="36" t="s">
+        <v>629</v>
+      </c>
+      <c r="E13" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F13" s="36" t="s">
+        <v>653</v>
+      </c>
+      <c r="G13" s="36"/>
+      <c r="H13" s="37"/>
+      <c r="I13" s="37"/>
+      <c r="J13" s="37"/>
+      <c r="K13" s="37"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="62" t="s">
+        <v>660</v>
+      </c>
+      <c r="B14" s="62" t="s">
+        <v>618</v>
+      </c>
+      <c r="C14" s="36" t="s">
+        <v>652</v>
+      </c>
+      <c r="D14" s="36" t="s">
+        <v>630</v>
+      </c>
+      <c r="E14" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F14" s="36" t="s">
+        <v>653</v>
+      </c>
+      <c r="G14" s="36"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="37"/>
+      <c r="J14" s="37"/>
+      <c r="K14" s="37"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="62" t="s">
+        <v>661</v>
+      </c>
+      <c r="B15" s="62" t="s">
+        <v>619</v>
+      </c>
+      <c r="C15" s="36" t="s">
+        <v>662</v>
+      </c>
+      <c r="D15" s="36" t="s">
+        <v>631</v>
+      </c>
+      <c r="E15" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F15" s="36" t="s">
+        <v>637</v>
+      </c>
+      <c r="G15" s="36"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="37"/>
+      <c r="K15" s="37"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="62" t="s">
+        <v>663</v>
+      </c>
+      <c r="B16" s="62" t="s">
+        <v>620</v>
+      </c>
+      <c r="C16" s="36" t="s">
+        <v>662</v>
+      </c>
+      <c r="D16" s="36" t="s">
+        <v>664</v>
+      </c>
+      <c r="E16" s="36" t="s">
+        <v>636</v>
+      </c>
+      <c r="F16" s="36" t="s">
+        <v>640</v>
+      </c>
+      <c r="G16" s="36"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="37"/>
+      <c r="K16" s="37"/>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="37"/>
+      <c r="K17" s="37"/>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" s="37"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="20" t="s">
+        <v>536</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>578</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>577</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>416</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>594</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" s="26"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="12"/>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="26"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="12"/>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" s="26"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="28" t="s">
+        <v>538</v>
+      </c>
+      <c r="F23" s="12"/>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="26"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="12"/>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="26"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="12"/>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="26"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="12"/>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="26"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="12"/>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="26"/>
+      <c r="B28" s="26" t="s">
+        <v>632</v>
+      </c>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="12"/>
+    </row>
+    <row r="29" spans="1:11" ht="119">
+      <c r="A29" s="26" t="s">
+        <v>633</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>585</v>
       </c>
-      <c r="B1" s="20" t="s">
-        <v>586</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>402</v>
-      </c>
-      <c r="D1" s="20" t="s">
-        <v>543</v>
-      </c>
-      <c r="E1" s="20" t="s">
-        <v>565</v>
-      </c>
-      <c r="F1" s="20" t="s">
-        <v>535</v>
-      </c>
-      <c r="G1" s="20" t="s">
-        <v>536</v>
-      </c>
-      <c r="H1" s="20" t="s">
-        <v>578</v>
-      </c>
-      <c r="I1" s="20" t="s">
-        <v>577</v>
-      </c>
-      <c r="J1" s="21" t="s">
-        <v>416</v>
-      </c>
-      <c r="K1" s="21" t="s">
-        <v>573</v>
-      </c>
-      <c r="L1" s="23" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="A2" s="25" t="s">
-        <v>487</v>
-      </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>545</v>
-      </c>
-      <c r="E2" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="12"/>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" s="25"/>
-      <c r="B3" s="25"/>
-      <c r="C3" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>545</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="12"/>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="25"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>545</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>537</v>
-      </c>
-      <c r="F4" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="28" t="s">
-        <v>538</v>
-      </c>
-      <c r="L4" s="12"/>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="25"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>545</v>
-      </c>
-      <c r="E5" s="26" t="s">
-        <v>4</v>
-      </c>
-      <c r="F5" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="12"/>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="25"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>545</v>
-      </c>
-      <c r="E6" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>362</v>
-      </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="12"/>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="25"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>545</v>
-      </c>
-      <c r="E7" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="12"/>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D8" s="26" t="s">
-        <v>545</v>
-      </c>
-      <c r="E8" s="28" t="s">
-        <v>360</v>
-      </c>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="26"/>
-      <c r="L8" s="12"/>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="D9" s="26" t="s">
-        <v>539</v>
-      </c>
-      <c r="E9" s="28" t="s">
-        <v>403</v>
-      </c>
-      <c r="F9" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="12"/>
-    </row>
-    <row r="10" spans="1:12" ht="119">
-      <c r="A10" s="25"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>539</v>
-      </c>
-      <c r="E10" s="28" t="s">
-        <v>403</v>
-      </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="13" t="s">
-        <v>584</v>
-      </c>
-      <c r="I10" s="13" t="s">
+      <c r="C29" s="13" t="s">
         <v>557</v>
       </c>
-      <c r="J10" s="17" t="s">
+      <c r="D29" s="17" t="s">
         <v>558</v>
       </c>
-      <c r="K10" s="12" t="s">
+      <c r="E29" s="12" t="s">
         <v>471</v>
       </c>
-      <c r="L10" s="12" t="s">
+      <c r="F29" s="12" t="s">
         <v>464</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" ht="102" customHeight="1">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>539</v>
-      </c>
-      <c r="E11" s="28" t="s">
-        <v>403</v>
-      </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="13" t="s">
-        <v>376</v>
-      </c>
-      <c r="I11" s="14" t="s">
+      <c r="I29" s="61" t="s">
+        <v>605</v>
+      </c>
+      <c r="J29" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="102">
+      <c r="A30" s="26"/>
+      <c r="B30" s="13" t="s">
+        <v>601</v>
+      </c>
+      <c r="C30" s="14" t="s">
         <v>377</v>
       </c>
-      <c r="J11" s="12" t="s">
+      <c r="D30" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="K11" s="12" t="s">
+      <c r="E30" s="12" t="s">
         <v>466</v>
       </c>
-      <c r="L11" s="12" t="s">
+      <c r="F30" s="12" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="153">
-      <c r="A12" s="25"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="D12" s="26" t="s">
-        <v>539</v>
-      </c>
-      <c r="E12" s="28" t="s">
-        <v>403</v>
-      </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="13" t="s">
-        <v>378</v>
-      </c>
-      <c r="I12" s="14" t="s">
+    <row r="31" spans="1:11" ht="153">
+      <c r="A31" s="26"/>
+      <c r="B31" s="13" t="s">
+        <v>602</v>
+      </c>
+      <c r="C31" s="14" t="s">
         <v>380</v>
       </c>
-      <c r="J12" s="12" t="s">
+      <c r="D31" s="12" t="s">
         <v>560</v>
       </c>
-      <c r="K12" s="12" t="s">
+      <c r="E31" s="12" t="s">
         <v>465</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="F31" s="12" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="170">
-      <c r="A13" s="25"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="D13" s="26" t="s">
-        <v>539</v>
-      </c>
-      <c r="E13" s="28" t="s">
-        <v>403</v>
-      </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="13" t="s">
-        <v>368</v>
-      </c>
-      <c r="I13" s="14" t="s">
+    <row r="32" spans="1:11" ht="170">
+      <c r="A32" s="26"/>
+      <c r="B32" s="13" t="s">
+        <v>603</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>379</v>
       </c>
-      <c r="J13" s="12" t="s">
+      <c r="D32" s="12" t="s">
         <v>561</v>
       </c>
-      <c r="K13" s="12" t="s">
+      <c r="E32" s="12" t="s">
         <v>468</v>
       </c>
-      <c r="L13" s="12" t="s">
+      <c r="F32" s="12" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="85">
-      <c r="A14" s="25"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="D14" s="26" t="s">
-        <v>539</v>
-      </c>
-      <c r="E14" s="28" t="s">
-        <v>403</v>
-      </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="14" t="s">
-        <v>373</v>
-      </c>
-      <c r="I14" s="19"/>
-      <c r="J14" s="12" t="s">
+    <row r="33" spans="1:6" ht="102">
+      <c r="A33" s="26"/>
+      <c r="B33" s="14" t="s">
+        <v>604</v>
+      </c>
+      <c r="C33" s="19"/>
+      <c r="D33" s="12" t="s">
         <v>562</v>
       </c>
-      <c r="K14" s="12" t="s">
+      <c r="E33" s="12" t="s">
         <v>467</v>
       </c>
-      <c r="L14" s="12" t="s">
+      <c r="F33" s="12" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
-      <c r="A15" s="25"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D15" s="28" t="s">
-        <v>547</v>
-      </c>
-      <c r="E15" s="28" t="s">
-        <v>552</v>
-      </c>
-      <c r="F15" s="26" t="s">
+    <row r="34" spans="1:6">
+      <c r="A34" s="26" t="s">
         <v>555</v>
       </c>
-      <c r="G15" s="26" t="s">
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="28" t="s">
+        <v>556</v>
+      </c>
+      <c r="F34" s="27"/>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="26" t="s">
         <v>555</v>
       </c>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="28" t="s">
+      <c r="B35" s="26"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="28" t="s">
         <v>556</v>
       </c>
-      <c r="L15" s="27"/>
-    </row>
-    <row r="16" spans="1:12">
-      <c r="A16" s="25"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>546</v>
-      </c>
-      <c r="E16" s="28" t="s">
-        <v>554</v>
-      </c>
-      <c r="F16" s="26" t="s">
+      <c r="F35" s="27"/>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="26" t="s">
         <v>555</v>
       </c>
-      <c r="G16" s="26" t="s">
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="28" t="s">
+        <v>556</v>
+      </c>
+      <c r="F36" s="27"/>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="26" t="s">
         <v>555</v>
       </c>
-      <c r="H16" s="26"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="28" t="s">
+      <c r="B37" s="26"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="28" t="s">
         <v>556</v>
       </c>
-      <c r="L16" s="27"/>
-    </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="25"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D17" s="28" t="s">
-        <v>551</v>
-      </c>
-      <c r="E17" s="28" t="s">
-        <v>411</v>
-      </c>
-      <c r="F17" s="26" t="s">
+      <c r="F37" s="27"/>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="26" t="s">
         <v>555</v>
       </c>
-      <c r="G17" s="26" t="s">
+      <c r="B38" s="26"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="28" t="s">
+        <v>556</v>
+      </c>
+      <c r="F38" s="27"/>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="26" t="s">
         <v>555</v>
       </c>
-      <c r="H17" s="26"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="28" t="s">
+      <c r="B39" s="26"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="28" t="s">
         <v>556</v>
       </c>
-      <c r="L17" s="27"/>
-    </row>
-    <row r="18" spans="1:12">
-      <c r="A18" s="25"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D18" s="28" t="s">
-        <v>548</v>
-      </c>
-      <c r="E18" s="26" t="s">
-        <v>412</v>
-      </c>
-      <c r="F18" s="26" t="s">
+      <c r="F39" s="27"/>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="26" t="s">
         <v>555</v>
       </c>
-      <c r="G18" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="28" t="s">
+      <c r="B40" s="26"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="28" t="s">
         <v>556</v>
       </c>
-      <c r="L18" s="27"/>
-    </row>
-    <row r="19" spans="1:12">
-      <c r="A19" s="25"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>550</v>
-      </c>
-      <c r="E19" s="26" t="s">
-        <v>413</v>
-      </c>
-      <c r="F19" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="G19" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="26"/>
-      <c r="K19" s="28" t="s">
-        <v>556</v>
-      </c>
-      <c r="L19" s="27"/>
-    </row>
-    <row r="20" spans="1:12">
-      <c r="A20" s="25"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>549</v>
-      </c>
-      <c r="E20" s="26" t="s">
-        <v>414</v>
-      </c>
-      <c r="F20" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="G20" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="28" t="s">
-        <v>556</v>
-      </c>
-      <c r="L20" s="27"/>
-    </row>
-    <row r="21" spans="1:12">
-      <c r="A21" s="25"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="26" t="s">
-        <v>404</v>
-      </c>
-      <c r="D21" s="28" t="s">
-        <v>549</v>
-      </c>
-      <c r="E21" s="26" t="s">
-        <v>415</v>
-      </c>
-      <c r="F21" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="G21" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="H21" s="26"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="28" t="s">
-        <v>556</v>
-      </c>
-      <c r="L21" s="27"/>
+      <c r="F40" s="27"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A1:B2 C1:L21">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="TBD">
-      <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
+  <conditionalFormatting sqref="A20:F40">
+    <cfRule type="containsText" dxfId="63" priority="3" operator="containsText" text="TBD">
+      <formula>NOT(ISERROR(SEARCH("TBD",A20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31611,10 +32350,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>408</v>
+        <v>586</v>
       </c>
       <c r="G1" s="22" t="s">
         <v>576</v>
@@ -31649,7 +32388,7 @@
         <v>473</v>
       </c>
       <c r="F2" s="39" t="s">
-        <v>567</v>
+        <v>593</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>20</v>
@@ -31718,7 +32457,7 @@
         <v>474</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>486</v>
+        <v>596</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>31</v>
@@ -35786,6 +36525,7 @@
       <c r="J216" s="27"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K1" xr:uid="{64F9033C-925C-4ABA-B39C-3AB8DF7B0920}"/>
   <mergeCells count="223">
     <mergeCell ref="I137:I141"/>
     <mergeCell ref="A137:A141"/>
@@ -36013,62 +36753,62 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:D26 G1:K26 A43:D141 G35:K141">
-    <cfRule type="containsText" dxfId="13" priority="12" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="60" priority="12" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:D27 B28:D34 G27:K34">
-    <cfRule type="containsText" dxfId="12" priority="11" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="59" priority="11" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E26 E43:E50">
-    <cfRule type="containsText" dxfId="11" priority="10" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="58" priority="10" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27">
-    <cfRule type="containsText" dxfId="10" priority="9" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="57" priority="9" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="containsText" dxfId="9" priority="8" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="56" priority="8" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E51:E68">
-    <cfRule type="containsText" dxfId="8" priority="7" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="55" priority="7" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E51)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E69:E90">
-    <cfRule type="containsText" dxfId="7" priority="6" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="54" priority="6" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E69)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E91:E115">
-    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="53" priority="5" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E91)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E116 E122:E141">
-    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="52" priority="4" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E116)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E119">
-    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="51" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E119)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F26 F35:F141">
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="50" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F27:F34">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="49" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",F27)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -36387,17 +37127,17 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="D5:D7">
-    <cfRule type="containsText" dxfId="16" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="48" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D3">
-    <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="47" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D4">
-    <cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="46" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D4)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -36430,14 +37170,16 @@
         <v>574</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="25" t="s">
-        <v>572</v>
-      </c>
-      <c r="B2" s="25"/>
+        <v>598</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>597</v>
+      </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="25" t="s">
@@ -36827,47 +37569,47 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="B1:B21">
-    <cfRule type="containsText" dxfId="25" priority="9" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="45" priority="9" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",B1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A21">
-    <cfRule type="containsText" dxfId="24" priority="8" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="44" priority="8" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="containsText" dxfId="23" priority="6" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="43" priority="6" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A25:C45">
-    <cfRule type="containsText" dxfId="22" priority="7" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="42" priority="7" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A25)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="containsText" dxfId="21" priority="5" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="41" priority="5" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",B49)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C49">
-    <cfRule type="containsText" dxfId="20" priority="4" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="40" priority="4" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",C49)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D49">
-    <cfRule type="containsText" dxfId="19" priority="3" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="39" priority="3" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D49)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A49">
-    <cfRule type="containsText" dxfId="18" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="38" priority="2" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",A49)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="containsText" dxfId="17" priority="1" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="37" priority="1" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",D1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>